<commit_message>
feat(hedgeye): 3-tier poll schedule, note-only panel dates, backfill hardening
- 3-tier Hedgeye poll cadence matching observed email send-time clustering:
  5 min (6:00-10:30am), 15 min (10:30am-4pm), 60 min otherwise. Quiet the
  "0 emails processed" poll log to DEBUG.
- Early Look / Call Macro Commentary panel cards no longer wait on the
  market-close anchor to advance -- same-day notes show immediately when
  viewing live, while historical date views stay capped at that date
  (no look-ahead), mirroring drv_quote's rule in derive_date_logic.md.
- RR/Call/ETFChange/IIChange parser + dispatch fixes, MSR gamma-throttle OCR
  hardening, panel/nav layout updates, new backfill/purge utility scripts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etl/working/ETFChange 2026-06-01.xlsx
+++ b/etl/working/ETFChange 2026-06-01.xlsx
@@ -16,11 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,31 +27,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-        <bgColor rgb="00FFFF99"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,25 +44,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,79 +420,79 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t xml:space="preserve"> Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t xml:space="preserve"> Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t xml:space="preserve"> Outlook</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t xml:space="preserve"> Action</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Aerospace &amp; Defense</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>XAR</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Long</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>add</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Social Media (SOCL) -</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Social Media</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>SOCL</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Neutral</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>remove</t>
         </is>
       </c>
     </row>

</xml_diff>